<commit_message>
Add reward config loading and standardize recipe craft times
</commit_message>
<xml_diff>
--- a/config/xlsx/recipes.xlsx
+++ b/config/xlsx/recipes.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="recipes" sheetId="1" r:id="R55a2cb734af34506"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="recipes" sheetId="1" r:id="R6035760237fc4dc4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -419,7 +419,7 @@
         <x:v>27001</x:v>
       </x:c>
       <x:c r="E2" s="3" t="n">
-        <x:v>15</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -440,7 +440,7 @@
         <x:v>27002</x:v>
       </x:c>
       <x:c r="E3" s="3" t="n">
-        <x:v>15</x:v>
+        <x:v>180</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -461,7 +461,7 @@
         <x:v>27003</x:v>
       </x:c>
       <x:c r="E4" s="3" t="n">
-        <x:v>15</x:v>
+        <x:v>300</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -482,7 +482,7 @@
         <x:v>27004</x:v>
       </x:c>
       <x:c r="E5" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>600</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -503,7 +503,7 @@
         <x:v>27005</x:v>
       </x:c>
       <x:c r="E6" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>1200</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -524,7 +524,7 @@
         <x:v>27006</x:v>
       </x:c>
       <x:c r="E7" s="3" t="n">
-        <x:v>15</x:v>
+        <x:v>600</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -545,7 +545,7 @@
         <x:v>27007</x:v>
       </x:c>
       <x:c r="E8" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>1200</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -566,7 +566,7 @@
         <x:v>27008</x:v>
       </x:c>
       <x:c r="E9" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>1800</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -587,7 +587,7 @@
         <x:v>27009</x:v>
       </x:c>
       <x:c r="E10" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>2700</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -608,7 +608,7 @@
         <x:v>27010</x:v>
       </x:c>
       <x:c r="E11" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>3600</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -629,7 +629,7 @@
         <x:v>27011</x:v>
       </x:c>
       <x:c r="E12" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>5400</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -650,7 +650,7 @@
         <x:v>27012</x:v>
       </x:c>
       <x:c r="E13" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>7200</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -671,7 +671,7 @@
         <x:v>27013</x:v>
       </x:c>
       <x:c r="E14" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>10800</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -692,7 +692,7 @@
         <x:v>27014</x:v>
       </x:c>
       <x:c r="E15" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>14400</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -713,7 +713,7 @@
         <x:v>27015</x:v>
       </x:c>
       <x:c r="E16" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>5400</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -734,7 +734,7 @@
         <x:v>27016</x:v>
       </x:c>
       <x:c r="E17" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>7200</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -755,7 +755,7 @@
         <x:v>27017</x:v>
       </x:c>
       <x:c r="E18" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>10800</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -776,7 +776,7 @@
         <x:v>27018</x:v>
       </x:c>
       <x:c r="E19" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>14400</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -797,7 +797,7 @@
         <x:v>27019</x:v>
       </x:c>
       <x:c r="E20" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>14400</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -818,7 +818,7 @@
         <x:v>27020</x:v>
       </x:c>
       <x:c r="E21" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>10800</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -839,7 +839,7 @@
         <x:v>27021</x:v>
       </x:c>
       <x:c r="E22" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>10800</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -860,7 +860,7 @@
         <x:v>27022</x:v>
       </x:c>
       <x:c r="E23" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>14400</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -881,7 +881,7 @@
         <x:v>27023</x:v>
       </x:c>
       <x:c r="E24" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>21600</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -902,7 +902,7 @@
         <x:v>27024</x:v>
       </x:c>
       <x:c r="E25" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>28800</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -923,7 +923,7 @@
         <x:v>27025</x:v>
       </x:c>
       <x:c r="E26" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>36000</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -944,7 +944,7 @@
         <x:v>27026</x:v>
       </x:c>
       <x:c r="E27" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>43200</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -965,7 +965,7 @@
         <x:v>27027</x:v>
       </x:c>
       <x:c r="E28" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>21600</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -986,7 +986,7 @@
         <x:v>27028</x:v>
       </x:c>
       <x:c r="E29" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>28800</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -1007,7 +1007,7 @@
         <x:v>27029</x:v>
       </x:c>
       <x:c r="E30" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>36000</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -1028,7 +1028,7 @@
         <x:v>27030</x:v>
       </x:c>
       <x:c r="E31" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>43200</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -1049,7 +1049,7 @@
         <x:v>27031</x:v>
       </x:c>
       <x:c r="E32" s="3" t="n">
-        <x:v>15</x:v>
+        <x:v>600</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -1070,7 +1070,7 @@
         <x:v>27081</x:v>
       </x:c>
       <x:c r="E33" s="3" t="n">
-        <x:v>15</x:v>
+        <x:v>600</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -1091,7 +1091,7 @@
         <x:v>27033</x:v>
       </x:c>
       <x:c r="E34" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>600</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -1112,7 +1112,7 @@
         <x:v>27034</x:v>
       </x:c>
       <x:c r="E35" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>1200</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -1133,7 +1133,7 @@
         <x:v>27035</x:v>
       </x:c>
       <x:c r="E36" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>1800</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -1154,7 +1154,7 @@
         <x:v>27036</x:v>
       </x:c>
       <x:c r="E37" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>2700</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -1175,7 +1175,7 @@
         <x:v>27037</x:v>
       </x:c>
       <x:c r="E38" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>3600</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -1196,7 +1196,7 @@
         <x:v>27038</x:v>
       </x:c>
       <x:c r="E39" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>5400</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -1217,7 +1217,7 @@
         <x:v>27039</x:v>
       </x:c>
       <x:c r="E40" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>7200</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -1238,7 +1238,7 @@
         <x:v>27040</x:v>
       </x:c>
       <x:c r="E41" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>10800</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -1259,7 +1259,7 @@
         <x:v>27041</x:v>
       </x:c>
       <x:c r="E42" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>14400</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -1280,7 +1280,7 @@
         <x:v>27042</x:v>
       </x:c>
       <x:c r="E43" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>21600</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -1301,7 +1301,7 @@
         <x:v>27043</x:v>
       </x:c>
       <x:c r="E44" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>28800</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -1322,7 +1322,7 @@
         <x:v>27044</x:v>
       </x:c>
       <x:c r="E45" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>36000</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -1343,7 +1343,7 @@
         <x:v>27045</x:v>
       </x:c>
       <x:c r="E46" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>43200</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -1364,7 +1364,7 @@
         <x:v>27046</x:v>
       </x:c>
       <x:c r="E47" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>43200</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -1385,7 +1385,7 @@
         <x:v>27047</x:v>
       </x:c>
       <x:c r="E48" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>43200</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -1406,7 +1406,7 @@
         <x:v>27048</x:v>
       </x:c>
       <x:c r="E49" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>43200</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -1427,7 +1427,7 @@
         <x:v>27049</x:v>
       </x:c>
       <x:c r="E50" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>10800</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -1448,7 +1448,7 @@
         <x:v>27050</x:v>
       </x:c>
       <x:c r="E51" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>43200</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -1469,7 +1469,7 @@
         <x:v>27051</x:v>
       </x:c>
       <x:c r="E52" s="3" t="n">
-        <x:v>15</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
@@ -1490,7 +1490,7 @@
         <x:v>27052</x:v>
       </x:c>
       <x:c r="E53" s="3" t="n">
-        <x:v>15</x:v>
+        <x:v>180</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -1511,7 +1511,7 @@
         <x:v>27053</x:v>
       </x:c>
       <x:c r="E54" s="3" t="n">
-        <x:v>15</x:v>
+        <x:v>300</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
@@ -1532,7 +1532,7 @@
         <x:v>27054</x:v>
       </x:c>
       <x:c r="E55" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>600</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -1553,7 +1553,7 @@
         <x:v>27055</x:v>
       </x:c>
       <x:c r="E56" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>1200</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
@@ -1574,7 +1574,7 @@
         <x:v>27056</x:v>
       </x:c>
       <x:c r="E57" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>1800</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
@@ -1595,7 +1595,7 @@
         <x:v>27057</x:v>
       </x:c>
       <x:c r="E58" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>2700</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
@@ -1616,7 +1616,7 @@
         <x:v>27058</x:v>
       </x:c>
       <x:c r="E59" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>3600</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
@@ -1637,7 +1637,7 @@
         <x:v>27059</x:v>
       </x:c>
       <x:c r="E60" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>5400</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
@@ -1658,7 +1658,7 @@
         <x:v>27060</x:v>
       </x:c>
       <x:c r="E61" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>7200</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
@@ -1679,7 +1679,7 @@
         <x:v>27061</x:v>
       </x:c>
       <x:c r="E62" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>1200</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
@@ -1700,7 +1700,7 @@
         <x:v>27062</x:v>
       </x:c>
       <x:c r="E63" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>1800</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
@@ -1721,7 +1721,7 @@
         <x:v>27063</x:v>
       </x:c>
       <x:c r="E64" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>2700</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
@@ -1742,7 +1742,7 @@
         <x:v>27064</x:v>
       </x:c>
       <x:c r="E65" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>3600</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
@@ -1763,7 +1763,7 @@
         <x:v>27065</x:v>
       </x:c>
       <x:c r="E66" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>5400</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
@@ -1784,7 +1784,7 @@
         <x:v>27066</x:v>
       </x:c>
       <x:c r="E67" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>7200</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
@@ -1805,7 +1805,7 @@
         <x:v>27067</x:v>
       </x:c>
       <x:c r="E68" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>10800</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
@@ -1826,7 +1826,7 @@
         <x:v>27068</x:v>
       </x:c>
       <x:c r="E69" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>14400</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
@@ -1847,7 +1847,7 @@
         <x:v>27069</x:v>
       </x:c>
       <x:c r="E70" s="3" t="n">
-        <x:v>15</x:v>
+        <x:v>5400</x:v>
       </x:c>
     </x:row>
     <x:row r="71">
@@ -1868,7 +1868,7 @@
         <x:v>27070</x:v>
       </x:c>
       <x:c r="E71" s="3" t="n">
-        <x:v>15</x:v>
+        <x:v>7200</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
@@ -1889,7 +1889,7 @@
         <x:v>27071</x:v>
       </x:c>
       <x:c r="E72" s="3" t="n">
-        <x:v>15</x:v>
+        <x:v>10800</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
@@ -1910,7 +1910,7 @@
         <x:v>27072</x:v>
       </x:c>
       <x:c r="E73" s="3" t="n">
-        <x:v>15</x:v>
+        <x:v>14400</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
@@ -1931,7 +1931,7 @@
         <x:v>27073</x:v>
       </x:c>
       <x:c r="E74" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>21600</x:v>
       </x:c>
     </x:row>
     <x:row r="75">
@@ -1952,7 +1952,7 @@
         <x:v>27074</x:v>
       </x:c>
       <x:c r="E75" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>28800</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
@@ -1973,7 +1973,7 @@
         <x:v>27075</x:v>
       </x:c>
       <x:c r="E76" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>36000</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
@@ -1994,7 +1994,7 @@
         <x:v>27080</x:v>
       </x:c>
       <x:c r="E77" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>43200</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
@@ -2015,7 +2015,7 @@
         <x:v>27077</x:v>
       </x:c>
       <x:c r="E78" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>21600</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
@@ -2036,7 +2036,7 @@
         <x:v>27078</x:v>
       </x:c>
       <x:c r="E79" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>28800</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
@@ -2057,7 +2057,7 @@
         <x:v>27079</x:v>
       </x:c>
       <x:c r="E80" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>36000</x:v>
       </x:c>
     </x:row>
     <x:row r="81">
@@ -2078,7 +2078,7 @@
         <x:v>27080</x:v>
       </x:c>
       <x:c r="E81" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>43200</x:v>
       </x:c>
     </x:row>
     <x:row r="82">
@@ -2099,7 +2099,7 @@
         <x:v>27081</x:v>
       </x:c>
       <x:c r="E82" s="3" t="n">
-        <x:v>15</x:v>
+        <x:v>600</x:v>
       </x:c>
     </x:row>
     <x:row r="83">
@@ -2120,7 +2120,7 @@
         <x:v>27082</x:v>
       </x:c>
       <x:c r="E83" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>600</x:v>
       </x:c>
     </x:row>
     <x:row r="84">
@@ -2141,7 +2141,7 @@
         <x:v>27083</x:v>
       </x:c>
       <x:c r="E84" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>1200</x:v>
       </x:c>
     </x:row>
     <x:row r="85">
@@ -2162,7 +2162,7 @@
         <x:v>27084</x:v>
       </x:c>
       <x:c r="E85" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>1800</x:v>
       </x:c>
     </x:row>
     <x:row r="86">
@@ -2183,7 +2183,7 @@
         <x:v>27085</x:v>
       </x:c>
       <x:c r="E86" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>2700</x:v>
       </x:c>
     </x:row>
     <x:row r="87">
@@ -2204,7 +2204,7 @@
         <x:v>27086</x:v>
       </x:c>
       <x:c r="E87" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>3600</x:v>
       </x:c>
     </x:row>
     <x:row r="88">
@@ -2225,7 +2225,7 @@
         <x:v>27087</x:v>
       </x:c>
       <x:c r="E88" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>5400</x:v>
       </x:c>
     </x:row>
     <x:row r="89">
@@ -2246,7 +2246,7 @@
         <x:v>27088</x:v>
       </x:c>
       <x:c r="E89" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>7200</x:v>
       </x:c>
     </x:row>
     <x:row r="90">
@@ -2267,7 +2267,7 @@
         <x:v>27089</x:v>
       </x:c>
       <x:c r="E90" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>10800</x:v>
       </x:c>
     </x:row>
     <x:row r="91">
@@ -2288,7 +2288,7 @@
         <x:v>27090</x:v>
       </x:c>
       <x:c r="E91" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>14400</x:v>
       </x:c>
     </x:row>
     <x:row r="92">
@@ -2309,7 +2309,7 @@
         <x:v>27091</x:v>
       </x:c>
       <x:c r="E92" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>21600</x:v>
       </x:c>
     </x:row>
     <x:row r="93">
@@ -2330,7 +2330,7 @@
         <x:v>27092</x:v>
       </x:c>
       <x:c r="E93" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>28800</x:v>
       </x:c>
     </x:row>
     <x:row r="94">
@@ -2351,7 +2351,7 @@
         <x:v>27093</x:v>
       </x:c>
       <x:c r="E94" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>36000</x:v>
       </x:c>
     </x:row>
     <x:row r="95">
@@ -2372,7 +2372,7 @@
         <x:v>27094</x:v>
       </x:c>
       <x:c r="E95" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>43200</x:v>
       </x:c>
     </x:row>
     <x:row r="96">
@@ -2393,7 +2393,7 @@
         <x:v>27095</x:v>
       </x:c>
       <x:c r="E96" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>14400</x:v>
       </x:c>
     </x:row>
     <x:row r="97">
@@ -2414,7 +2414,7 @@
         <x:v>27096</x:v>
       </x:c>
       <x:c r="E97" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>43200</x:v>
       </x:c>
     </x:row>
     <x:row r="98">
@@ -2435,7 +2435,7 @@
         <x:v>27097</x:v>
       </x:c>
       <x:c r="E98" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>7200</x:v>
       </x:c>
     </x:row>
     <x:row r="99">
@@ -2456,7 +2456,7 @@
         <x:v>27099</x:v>
       </x:c>
       <x:c r="E99" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>43200</x:v>
       </x:c>
     </x:row>
     <x:row r="100">
@@ -2477,7 +2477,7 @@
         <x:v>27100</x:v>
       </x:c>
       <x:c r="E100" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>43200</x:v>
       </x:c>
     </x:row>
     <x:row r="101">
@@ -2498,7 +2498,7 @@
         <x:v>27101</x:v>
       </x:c>
       <x:c r="E101" s="3" t="n">
-        <x:v>15</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="102">
@@ -2519,7 +2519,7 @@
         <x:v>27102</x:v>
       </x:c>
       <x:c r="E102" s="3" t="n">
-        <x:v>15</x:v>
+        <x:v>180</x:v>
       </x:c>
     </x:row>
     <x:row r="103">
@@ -2540,7 +2540,7 @@
         <x:v>27103</x:v>
       </x:c>
       <x:c r="E103" s="3" t="n">
-        <x:v>15</x:v>
+        <x:v>300</x:v>
       </x:c>
     </x:row>
     <x:row r="104">
@@ -2561,7 +2561,7 @@
         <x:v>27104</x:v>
       </x:c>
       <x:c r="E104" s="3" t="n">
-        <x:v>15</x:v>
+        <x:v>600</x:v>
       </x:c>
     </x:row>
     <x:row r="105">
@@ -2582,7 +2582,7 @@
         <x:v>27105</x:v>
       </x:c>
       <x:c r="E105" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>300</x:v>
       </x:c>
     </x:row>
     <x:row r="106">
@@ -2603,7 +2603,7 @@
         <x:v>27106</x:v>
       </x:c>
       <x:c r="E106" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>1200</x:v>
       </x:c>
     </x:row>
     <x:row r="107">
@@ -2624,7 +2624,7 @@
         <x:v>27107</x:v>
       </x:c>
       <x:c r="E107" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>1800</x:v>
       </x:c>
     </x:row>
     <x:row r="108">
@@ -2645,7 +2645,7 @@
         <x:v>27108</x:v>
       </x:c>
       <x:c r="E108" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>2700</x:v>
       </x:c>
     </x:row>
     <x:row r="109">
@@ -2666,7 +2666,7 @@
         <x:v>27109</x:v>
       </x:c>
       <x:c r="E109" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>3600</x:v>
       </x:c>
     </x:row>
     <x:row r="110">
@@ -2687,7 +2687,7 @@
         <x:v>27110</x:v>
       </x:c>
       <x:c r="E110" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>5400</x:v>
       </x:c>
     </x:row>
     <x:row r="111">
@@ -2708,7 +2708,7 @@
         <x:v>27111</x:v>
       </x:c>
       <x:c r="E111" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>7200</x:v>
       </x:c>
     </x:row>
     <x:row r="112">
@@ -2729,7 +2729,7 @@
         <x:v>27112</x:v>
       </x:c>
       <x:c r="E112" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>10800</x:v>
       </x:c>
     </x:row>
     <x:row r="113">
@@ -2750,7 +2750,7 @@
         <x:v>27113</x:v>
       </x:c>
       <x:c r="E113" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>14400</x:v>
       </x:c>
     </x:row>
     <x:row r="114">
@@ -2771,7 +2771,7 @@
         <x:v>27114</x:v>
       </x:c>
       <x:c r="E114" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>21600</x:v>
       </x:c>
     </x:row>
     <x:row r="115">
@@ -2792,7 +2792,7 @@
         <x:v>27115</x:v>
       </x:c>
       <x:c r="E115" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>28800</x:v>
       </x:c>
     </x:row>
     <x:row r="116">
@@ -2813,7 +2813,7 @@
         <x:v>27116</x:v>
       </x:c>
       <x:c r="E116" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>36000</x:v>
       </x:c>
     </x:row>
     <x:row r="117">
@@ -2834,7 +2834,7 @@
         <x:v>27117</x:v>
       </x:c>
       <x:c r="E117" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>43200</x:v>
       </x:c>
     </x:row>
     <x:row r="118">
@@ -2855,7 +2855,7 @@
         <x:v>27118</x:v>
       </x:c>
       <x:c r="E118" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>1200</x:v>
       </x:c>
     </x:row>
     <x:row r="119">
@@ -2876,7 +2876,7 @@
         <x:v>27119</x:v>
       </x:c>
       <x:c r="E119" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>1800</x:v>
       </x:c>
     </x:row>
     <x:row r="120">
@@ -2897,7 +2897,7 @@
         <x:v>27120</x:v>
       </x:c>
       <x:c r="E120" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>2700</x:v>
       </x:c>
     </x:row>
     <x:row r="121">
@@ -2918,7 +2918,7 @@
         <x:v>27121</x:v>
       </x:c>
       <x:c r="E121" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>3600</x:v>
       </x:c>
     </x:row>
     <x:row r="122">
@@ -2939,7 +2939,7 @@
         <x:v>27122</x:v>
       </x:c>
       <x:c r="E122" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>5400</x:v>
       </x:c>
     </x:row>
     <x:row r="123">
@@ -2960,7 +2960,7 @@
         <x:v>27123</x:v>
       </x:c>
       <x:c r="E123" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>7200</x:v>
       </x:c>
     </x:row>
     <x:row r="124">
@@ -2981,7 +2981,7 @@
         <x:v>27124</x:v>
       </x:c>
       <x:c r="E124" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>10800</x:v>
       </x:c>
     </x:row>
     <x:row r="125">
@@ -3002,7 +3002,7 @@
         <x:v>27125</x:v>
       </x:c>
       <x:c r="E125" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>14400</x:v>
       </x:c>
     </x:row>
     <x:row r="126">
@@ -3023,7 +3023,7 @@
         <x:v>27126</x:v>
       </x:c>
       <x:c r="E126" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>21600</x:v>
       </x:c>
     </x:row>
     <x:row r="127">
@@ -3044,7 +3044,7 @@
         <x:v>27127</x:v>
       </x:c>
       <x:c r="E127" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>28800</x:v>
       </x:c>
     </x:row>
     <x:row r="128">
@@ -3065,7 +3065,7 @@
         <x:v>27128</x:v>
       </x:c>
       <x:c r="E128" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>36000</x:v>
       </x:c>
     </x:row>
     <x:row r="129">
@@ -3086,7 +3086,7 @@
         <x:v>27129</x:v>
       </x:c>
       <x:c r="E129" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>43200</x:v>
       </x:c>
     </x:row>
     <x:row r="130">
@@ -3107,7 +3107,7 @@
         <x:v>27130</x:v>
       </x:c>
       <x:c r="E130" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>600</x:v>
       </x:c>
     </x:row>
     <x:row r="131">
@@ -3128,7 +3128,7 @@
         <x:v>27131</x:v>
       </x:c>
       <x:c r="E131" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>5400</x:v>
       </x:c>
     </x:row>
     <x:row r="132">
@@ -3149,7 +3149,7 @@
         <x:v>27132</x:v>
       </x:c>
       <x:c r="E132" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>7200</x:v>
       </x:c>
     </x:row>
     <x:row r="133">
@@ -3170,7 +3170,7 @@
         <x:v>27133</x:v>
       </x:c>
       <x:c r="E133" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>10800</x:v>
       </x:c>
     </x:row>
     <x:row r="134">
@@ -3191,7 +3191,7 @@
         <x:v>27134</x:v>
       </x:c>
       <x:c r="E134" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>14400</x:v>
       </x:c>
     </x:row>
     <x:row r="135">
@@ -3212,7 +3212,7 @@
         <x:v>27135</x:v>
       </x:c>
       <x:c r="E135" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>21600</x:v>
       </x:c>
     </x:row>
     <x:row r="136">
@@ -3233,7 +3233,7 @@
         <x:v>27136</x:v>
       </x:c>
       <x:c r="E136" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>28800</x:v>
       </x:c>
     </x:row>
     <x:row r="137">
@@ -3254,7 +3254,7 @@
         <x:v>27137</x:v>
       </x:c>
       <x:c r="E137" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>36000</x:v>
       </x:c>
     </x:row>
     <x:row r="138">
@@ -3275,7 +3275,7 @@
         <x:v>27138</x:v>
       </x:c>
       <x:c r="E138" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>43200</x:v>
       </x:c>
     </x:row>
     <x:row r="139">
@@ -3296,7 +3296,7 @@
         <x:v>27139</x:v>
       </x:c>
       <x:c r="E139" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>1200</x:v>
       </x:c>
     </x:row>
     <x:row r="140">
@@ -3317,7 +3317,7 @@
         <x:v>27140</x:v>
       </x:c>
       <x:c r="E140" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>1800</x:v>
       </x:c>
     </x:row>
     <x:row r="141">
@@ -3338,7 +3338,7 @@
         <x:v>27141</x:v>
       </x:c>
       <x:c r="E141" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>2700</x:v>
       </x:c>
     </x:row>
     <x:row r="142">
@@ -3359,7 +3359,7 @@
         <x:v>27142</x:v>
       </x:c>
       <x:c r="E142" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>3600</x:v>
       </x:c>
     </x:row>
     <x:row r="143">
@@ -3380,7 +3380,7 @@
         <x:v>27143</x:v>
       </x:c>
       <x:c r="E143" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>14400</x:v>
       </x:c>
     </x:row>
     <x:row r="144">
@@ -3401,7 +3401,7 @@
         <x:v>27144</x:v>
       </x:c>
       <x:c r="E144" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>600</x:v>
       </x:c>
     </x:row>
     <x:row r="145">
@@ -3422,7 +3422,7 @@
         <x:v>27145</x:v>
       </x:c>
       <x:c r="E145" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>7200</x:v>
       </x:c>
     </x:row>
     <x:row r="146">
@@ -3443,7 +3443,7 @@
         <x:v>27146</x:v>
       </x:c>
       <x:c r="E146" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>10800</x:v>
       </x:c>
     </x:row>
     <x:row r="147">
@@ -3464,7 +3464,7 @@
         <x:v>27147</x:v>
       </x:c>
       <x:c r="E147" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>3600</x:v>
       </x:c>
     </x:row>
     <x:row r="148">
@@ -3485,7 +3485,7 @@
         <x:v>27148</x:v>
       </x:c>
       <x:c r="E148" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>28800</x:v>
       </x:c>
     </x:row>
     <x:row r="149">
@@ -3506,7 +3506,7 @@
         <x:v>27149</x:v>
       </x:c>
       <x:c r="E149" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>36000</x:v>
       </x:c>
     </x:row>
     <x:row r="150">
@@ -3527,7 +3527,7 @@
         <x:v>27150</x:v>
       </x:c>
       <x:c r="E150" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>43200</x:v>
       </x:c>
     </x:row>
     <x:row r="151">
@@ -3548,7 +3548,7 @@
         <x:v>28001</x:v>
       </x:c>
       <x:c r="E151" s="3" t="n">
-        <x:v>15</x:v>
+        <x:v>180</x:v>
       </x:c>
     </x:row>
     <x:row r="152">
@@ -3569,7 +3569,7 @@
         <x:v>28002</x:v>
       </x:c>
       <x:c r="E152" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>300</x:v>
       </x:c>
     </x:row>
     <x:row r="153">
@@ -3590,7 +3590,7 @@
         <x:v>28003</x:v>
       </x:c>
       <x:c r="E153" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>600</x:v>
       </x:c>
     </x:row>
     <x:row r="154">
@@ -3611,7 +3611,7 @@
         <x:v>28004</x:v>
       </x:c>
       <x:c r="E154" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>600</x:v>
       </x:c>
     </x:row>
     <x:row r="155">
@@ -3632,7 +3632,7 @@
         <x:v>28005</x:v>
       </x:c>
       <x:c r="E155" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>1200</x:v>
       </x:c>
     </x:row>
     <x:row r="156">
@@ -3653,7 +3653,7 @@
         <x:v>28006</x:v>
       </x:c>
       <x:c r="E156" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>1800</x:v>
       </x:c>
     </x:row>
     <x:row r="157">
@@ -3674,7 +3674,7 @@
         <x:v>28007</x:v>
       </x:c>
       <x:c r="E157" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>2700</x:v>
       </x:c>
     </x:row>
     <x:row r="158">
@@ -3695,7 +3695,7 @@
         <x:v>28008</x:v>
       </x:c>
       <x:c r="E158" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>3600</x:v>
       </x:c>
     </x:row>
     <x:row r="159">
@@ -3716,7 +3716,7 @@
         <x:v>28009</x:v>
       </x:c>
       <x:c r="E159" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>5400</x:v>
       </x:c>
     </x:row>
     <x:row r="160">
@@ -3737,7 +3737,7 @@
         <x:v>28010</x:v>
       </x:c>
       <x:c r="E160" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>7200</x:v>
       </x:c>
     </x:row>
     <x:row r="161">
@@ -3758,7 +3758,7 @@
         <x:v>28011</x:v>
       </x:c>
       <x:c r="E161" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>10800</x:v>
       </x:c>
     </x:row>
     <x:row r="162">
@@ -3779,7 +3779,7 @@
         <x:v>28012</x:v>
       </x:c>
       <x:c r="E162" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>14400</x:v>
       </x:c>
     </x:row>
     <x:row r="163">
@@ -3800,7 +3800,7 @@
         <x:v>28013</x:v>
       </x:c>
       <x:c r="E163" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>21600</x:v>
       </x:c>
     </x:row>
     <x:row r="164">
@@ -3821,7 +3821,7 @@
         <x:v>28014</x:v>
       </x:c>
       <x:c r="E164" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>28800</x:v>
       </x:c>
     </x:row>
     <x:row r="165">
@@ -3842,7 +3842,7 @@
         <x:v>28015</x:v>
       </x:c>
       <x:c r="E165" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>36000</x:v>
       </x:c>
     </x:row>
     <x:row r="166">
@@ -3863,7 +3863,7 @@
         <x:v>28016</x:v>
       </x:c>
       <x:c r="E166" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>43200</x:v>
       </x:c>
     </x:row>
     <x:row r="167">
@@ -3884,7 +3884,7 @@
         <x:v>28017</x:v>
       </x:c>
       <x:c r="E167" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="168">
@@ -3905,7 +3905,7 @@
         <x:v>28018</x:v>
       </x:c>
       <x:c r="E168" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>180</x:v>
       </x:c>
     </x:row>
     <x:row r="169">
@@ -3926,7 +3926,7 @@
         <x:v>28019</x:v>
       </x:c>
       <x:c r="E169" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>300</x:v>
       </x:c>
     </x:row>
     <x:row r="170">
@@ -3947,7 +3947,7 @@
         <x:v>28020</x:v>
       </x:c>
       <x:c r="E170" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>600</x:v>
       </x:c>
     </x:row>
     <x:row r="171">
@@ -3968,7 +3968,7 @@
         <x:v>28021</x:v>
       </x:c>
       <x:c r="E171" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>1200</x:v>
       </x:c>
     </x:row>
     <x:row r="172">
@@ -3989,7 +3989,7 @@
         <x:v>28022</x:v>
       </x:c>
       <x:c r="E172" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>1800</x:v>
       </x:c>
     </x:row>
     <x:row r="173">
@@ -4010,7 +4010,7 @@
         <x:v>28023</x:v>
       </x:c>
       <x:c r="E173" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>2700</x:v>
       </x:c>
     </x:row>
     <x:row r="174">
@@ -4031,7 +4031,7 @@
         <x:v>28024</x:v>
       </x:c>
       <x:c r="E174" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>3600</x:v>
       </x:c>
     </x:row>
     <x:row r="175">
@@ -4052,7 +4052,7 @@
         <x:v>28025</x:v>
       </x:c>
       <x:c r="E175" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>5400</x:v>
       </x:c>
     </x:row>
     <x:row r="176">
@@ -4073,7 +4073,7 @@
         <x:v>28026</x:v>
       </x:c>
       <x:c r="E176" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>7200</x:v>
       </x:c>
     </x:row>
     <x:row r="177">
@@ -4094,7 +4094,7 @@
         <x:v>28027</x:v>
       </x:c>
       <x:c r="E177" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>10800</x:v>
       </x:c>
     </x:row>
     <x:row r="178">
@@ -4115,7 +4115,7 @@
         <x:v>28028</x:v>
       </x:c>
       <x:c r="E178" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>14400</x:v>
       </x:c>
     </x:row>
     <x:row r="179">
@@ -4136,7 +4136,7 @@
         <x:v>28029</x:v>
       </x:c>
       <x:c r="E179" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>21600</x:v>
       </x:c>
     </x:row>
     <x:row r="180">
@@ -4157,7 +4157,7 @@
         <x:v>28030</x:v>
       </x:c>
       <x:c r="E180" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>28800</x:v>
       </x:c>
     </x:row>
     <x:row r="181">
@@ -4178,7 +4178,7 @@
         <x:v>28031</x:v>
       </x:c>
       <x:c r="E181" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>36000</x:v>
       </x:c>
     </x:row>
     <x:row r="182">
@@ -4199,7 +4199,7 @@
         <x:v>28032</x:v>
       </x:c>
       <x:c r="E182" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>43200</x:v>
       </x:c>
     </x:row>
     <x:row r="183">
@@ -4220,7 +4220,7 @@
         <x:v>28033</x:v>
       </x:c>
       <x:c r="E183" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="184">
@@ -4241,7 +4241,7 @@
         <x:v>28034</x:v>
       </x:c>
       <x:c r="E184" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>180</x:v>
       </x:c>
     </x:row>
     <x:row r="185">
@@ -4262,7 +4262,7 @@
         <x:v>28035</x:v>
       </x:c>
       <x:c r="E185" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>300</x:v>
       </x:c>
     </x:row>
     <x:row r="186">
@@ -4283,7 +4283,7 @@
         <x:v>28036</x:v>
       </x:c>
       <x:c r="E186" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>600</x:v>
       </x:c>
     </x:row>
     <x:row r="187">
@@ -4304,7 +4304,7 @@
         <x:v>28037</x:v>
       </x:c>
       <x:c r="E187" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>1200</x:v>
       </x:c>
     </x:row>
     <x:row r="188">
@@ -4325,7 +4325,7 @@
         <x:v>28038</x:v>
       </x:c>
       <x:c r="E188" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>1800</x:v>
       </x:c>
     </x:row>
     <x:row r="189">
@@ -4346,7 +4346,7 @@
         <x:v>28039</x:v>
       </x:c>
       <x:c r="E189" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>2700</x:v>
       </x:c>
     </x:row>
     <x:row r="190">
@@ -4367,7 +4367,7 @@
         <x:v>28040</x:v>
       </x:c>
       <x:c r="E190" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>3600</x:v>
       </x:c>
     </x:row>
     <x:row r="191">
@@ -4388,7 +4388,7 @@
         <x:v>28041</x:v>
       </x:c>
       <x:c r="E191" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>5400</x:v>
       </x:c>
     </x:row>
     <x:row r="192">
@@ -4409,7 +4409,7 @@
         <x:v>28042</x:v>
       </x:c>
       <x:c r="E192" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>7200</x:v>
       </x:c>
     </x:row>
     <x:row r="193">
@@ -4430,7 +4430,7 @@
         <x:v>28043</x:v>
       </x:c>
       <x:c r="E193" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>10800</x:v>
       </x:c>
     </x:row>
     <x:row r="194">
@@ -4451,7 +4451,7 @@
         <x:v>28044</x:v>
       </x:c>
       <x:c r="E194" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>14400</x:v>
       </x:c>
     </x:row>
     <x:row r="195">
@@ -4472,7 +4472,7 @@
         <x:v>28045</x:v>
       </x:c>
       <x:c r="E195" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>21600</x:v>
       </x:c>
     </x:row>
     <x:row r="196">
@@ -4493,7 +4493,7 @@
         <x:v>28046</x:v>
       </x:c>
       <x:c r="E196" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>28800</x:v>
       </x:c>
     </x:row>
     <x:row r="197">
@@ -4514,7 +4514,7 @@
         <x:v>28047</x:v>
       </x:c>
       <x:c r="E197" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>36000</x:v>
       </x:c>
     </x:row>
     <x:row r="198">
@@ -4535,7 +4535,7 @@
         <x:v>28048</x:v>
       </x:c>
       <x:c r="E198" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>43200</x:v>
       </x:c>
     </x:row>
     <x:row r="199">
@@ -4556,7 +4556,7 @@
         <x:v>28049</x:v>
       </x:c>
       <x:c r="E199" s="3" t="n">
-        <x:v>20</x:v>
+        <x:v>180</x:v>
       </x:c>
     </x:row>
     <x:row r="200">
@@ -4577,7 +4577,7 @@
         <x:v>28050</x:v>
       </x:c>
       <x:c r="E200" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>600</x:v>
       </x:c>
     </x:row>
     <x:row r="201">
@@ -4598,7 +4598,7 @@
         <x:v>28051</x:v>
       </x:c>
       <x:c r="E201" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>1200</x:v>
       </x:c>
     </x:row>
     <x:row r="202">
@@ -4619,7 +4619,7 @@
         <x:v>28052</x:v>
       </x:c>
       <x:c r="E202" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>1800</x:v>
       </x:c>
     </x:row>
     <x:row r="203">
@@ -4640,7 +4640,7 @@
         <x:v>28053</x:v>
       </x:c>
       <x:c r="E203" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>3600</x:v>
       </x:c>
     </x:row>
     <x:row r="204">
@@ -4661,7 +4661,7 @@
         <x:v>28054</x:v>
       </x:c>
       <x:c r="E204" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>7200</x:v>
       </x:c>
     </x:row>
     <x:row r="205">
@@ -4682,7 +4682,7 @@
         <x:v>28055</x:v>
       </x:c>
       <x:c r="E205" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>10800</x:v>
       </x:c>
     </x:row>
     <x:row r="206">
@@ -4703,7 +4703,7 @@
         <x:v>28056</x:v>
       </x:c>
       <x:c r="E206" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>14400</x:v>
       </x:c>
     </x:row>
     <x:row r="207">
@@ -4724,7 +4724,7 @@
         <x:v>28057</x:v>
       </x:c>
       <x:c r="E207" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>14400</x:v>
       </x:c>
     </x:row>
     <x:row r="208">
@@ -4745,7 +4745,7 @@
         <x:v>28058</x:v>
       </x:c>
       <x:c r="E208" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>28800</x:v>
       </x:c>
     </x:row>
     <x:row r="209">
@@ -4766,7 +4766,7 @@
         <x:v>28059</x:v>
       </x:c>
       <x:c r="E209" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>36000</x:v>
       </x:c>
     </x:row>
     <x:row r="210">
@@ -4787,7 +4787,7 @@
         <x:v>28060</x:v>
       </x:c>
       <x:c r="E210" s="3" t="n">
-        <x:v>25</x:v>
+        <x:v>43200</x:v>
       </x:c>
     </x:row>
     <x:row r="211">
@@ -4804,7 +4804,7 @@
         <x:v>28101</x:v>
       </x:c>
       <x:c r="E211" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="212">
@@ -4821,7 +4821,7 @@
         <x:v>28102</x:v>
       </x:c>
       <x:c r="E212" s="4" t="n">
-        <x:v>15</x:v>
+        <x:v>180</x:v>
       </x:c>
     </x:row>
     <x:row r="213">
@@ -4838,7 +4838,7 @@
         <x:v>28103</x:v>
       </x:c>
       <x:c r="E213" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>600</x:v>
       </x:c>
     </x:row>
     <x:row r="214">
@@ -4855,7 +4855,7 @@
         <x:v>28104</x:v>
       </x:c>
       <x:c r="E214" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>1200</x:v>
       </x:c>
     </x:row>
     <x:row r="215">
@@ -4872,7 +4872,7 @@
         <x:v>28105</x:v>
       </x:c>
       <x:c r="E215" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>2700</x:v>
       </x:c>
     </x:row>
     <x:row r="216">
@@ -4889,7 +4889,7 @@
         <x:v>28106</x:v>
       </x:c>
       <x:c r="E216" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>3600</x:v>
       </x:c>
     </x:row>
     <x:row r="217">
@@ -4906,7 +4906,7 @@
         <x:v>28107</x:v>
       </x:c>
       <x:c r="E217" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>7200</x:v>
       </x:c>
     </x:row>
     <x:row r="218">
@@ -4923,7 +4923,7 @@
         <x:v>28108</x:v>
       </x:c>
       <x:c r="E218" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>14400</x:v>
       </x:c>
     </x:row>
     <x:row r="219">
@@ -4940,7 +4940,7 @@
         <x:v>28109</x:v>
       </x:c>
       <x:c r="E219" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>28800</x:v>
       </x:c>
     </x:row>
     <x:row r="220">
@@ -4957,7 +4957,7 @@
         <x:v>28110</x:v>
       </x:c>
       <x:c r="E220" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>43200</x:v>
       </x:c>
     </x:row>
     <x:row r="221">
@@ -4974,7 +4974,7 @@
         <x:v>28111</x:v>
       </x:c>
       <x:c r="E221" s="4" t="n">
-        <x:v>15</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="222">
@@ -4991,7 +4991,7 @@
         <x:v>28112</x:v>
       </x:c>
       <x:c r="E222" s="4" t="n">
-        <x:v>15</x:v>
+        <x:v>180</x:v>
       </x:c>
     </x:row>
     <x:row r="223">
@@ -5008,7 +5008,7 @@
         <x:v>28113</x:v>
       </x:c>
       <x:c r="E223" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>600</x:v>
       </x:c>
     </x:row>
     <x:row r="224">
@@ -5025,7 +5025,7 @@
         <x:v>28114</x:v>
       </x:c>
       <x:c r="E224" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>1200</x:v>
       </x:c>
     </x:row>
     <x:row r="225">
@@ -5042,7 +5042,7 @@
         <x:v>28115</x:v>
       </x:c>
       <x:c r="E225" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>2700</x:v>
       </x:c>
     </x:row>
     <x:row r="226">
@@ -5059,7 +5059,7 @@
         <x:v>28116</x:v>
       </x:c>
       <x:c r="E226" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>3600</x:v>
       </x:c>
     </x:row>
     <x:row r="227">
@@ -5076,7 +5076,7 @@
         <x:v>28117</x:v>
       </x:c>
       <x:c r="E227" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>7200</x:v>
       </x:c>
     </x:row>
     <x:row r="228">
@@ -5093,7 +5093,7 @@
         <x:v>28118</x:v>
       </x:c>
       <x:c r="E228" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>14400</x:v>
       </x:c>
     </x:row>
     <x:row r="229">
@@ -5110,7 +5110,7 @@
         <x:v>28119</x:v>
       </x:c>
       <x:c r="E229" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>28800</x:v>
       </x:c>
     </x:row>
     <x:row r="230">
@@ -5127,7 +5127,7 @@
         <x:v>28120</x:v>
       </x:c>
       <x:c r="E230" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>43200</x:v>
       </x:c>
     </x:row>
     <x:row r="231">
@@ -5144,7 +5144,7 @@
         <x:v>28121</x:v>
       </x:c>
       <x:c r="E231" s="4" t="n">
-        <x:v>15</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="232">
@@ -5161,7 +5161,7 @@
         <x:v>28122</x:v>
       </x:c>
       <x:c r="E232" s="4" t="n">
-        <x:v>15</x:v>
+        <x:v>180</x:v>
       </x:c>
     </x:row>
     <x:row r="233">
@@ -5178,7 +5178,7 @@
         <x:v>28123</x:v>
       </x:c>
       <x:c r="E233" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>600</x:v>
       </x:c>
     </x:row>
     <x:row r="234">
@@ -5195,7 +5195,7 @@
         <x:v>28124</x:v>
       </x:c>
       <x:c r="E234" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>1200</x:v>
       </x:c>
     </x:row>
     <x:row r="235">
@@ -5212,7 +5212,7 @@
         <x:v>28125</x:v>
       </x:c>
       <x:c r="E235" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>2700</x:v>
       </x:c>
     </x:row>
     <x:row r="236">
@@ -5229,7 +5229,7 @@
         <x:v>28126</x:v>
       </x:c>
       <x:c r="E236" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>3600</x:v>
       </x:c>
     </x:row>
     <x:row r="237">
@@ -5246,7 +5246,7 @@
         <x:v>28127</x:v>
       </x:c>
       <x:c r="E237" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>7200</x:v>
       </x:c>
     </x:row>
     <x:row r="238">
@@ -5263,7 +5263,7 @@
         <x:v>28128</x:v>
       </x:c>
       <x:c r="E238" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>14400</x:v>
       </x:c>
     </x:row>
     <x:row r="239">
@@ -5280,7 +5280,7 @@
         <x:v>28129</x:v>
       </x:c>
       <x:c r="E239" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>28800</x:v>
       </x:c>
     </x:row>
     <x:row r="240">
@@ -5297,7 +5297,7 @@
         <x:v>28130</x:v>
       </x:c>
       <x:c r="E240" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>43200</x:v>
       </x:c>
     </x:row>
     <x:row r="241">
@@ -5314,7 +5314,7 @@
         <x:v>28131</x:v>
       </x:c>
       <x:c r="E241" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="242">
@@ -5331,7 +5331,7 @@
         <x:v>28132</x:v>
       </x:c>
       <x:c r="E242" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>180</x:v>
       </x:c>
     </x:row>
     <x:row r="243">
@@ -5348,7 +5348,7 @@
         <x:v>28133</x:v>
       </x:c>
       <x:c r="E243" s="4" t="n">
-        <x:v>25</x:v>
+        <x:v>600</x:v>
       </x:c>
     </x:row>
     <x:row r="244">
@@ -5365,7 +5365,7 @@
         <x:v>28134</x:v>
       </x:c>
       <x:c r="E244" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>1200</x:v>
       </x:c>
     </x:row>
     <x:row r="245">
@@ -5382,7 +5382,7 @@
         <x:v>28135</x:v>
       </x:c>
       <x:c r="E245" s="4" t="n">
-        <x:v>25</x:v>
+        <x:v>2700</x:v>
       </x:c>
     </x:row>
     <x:row r="246">
@@ -5399,7 +5399,7 @@
         <x:v>28136</x:v>
       </x:c>
       <x:c r="E246" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>3600</x:v>
       </x:c>
     </x:row>
     <x:row r="247">
@@ -5416,7 +5416,7 @@
         <x:v>28137</x:v>
       </x:c>
       <x:c r="E247" s="4" t="n">
-        <x:v>25</x:v>
+        <x:v>7200</x:v>
       </x:c>
     </x:row>
     <x:row r="248">
@@ -5433,7 +5433,7 @@
         <x:v>28138</x:v>
       </x:c>
       <x:c r="E248" s="4" t="n">
-        <x:v>25</x:v>
+        <x:v>14400</x:v>
       </x:c>
     </x:row>
     <x:row r="249">
@@ -5450,7 +5450,7 @@
         <x:v>28139</x:v>
       </x:c>
       <x:c r="E249" s="4" t="n">
-        <x:v>25</x:v>
+        <x:v>28800</x:v>
       </x:c>
     </x:row>
     <x:row r="250">
@@ -5467,7 +5467,7 @@
         <x:v>28140</x:v>
       </x:c>
       <x:c r="E250" s="4" t="n">
-        <x:v>25</x:v>
+        <x:v>43200</x:v>
       </x:c>
     </x:row>
     <x:row r="251">
@@ -5484,7 +5484,7 @@
         <x:v>28141</x:v>
       </x:c>
       <x:c r="E251" s="4" t="n">
-        <x:v>15</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="252">
@@ -5501,7 +5501,7 @@
         <x:v>28142</x:v>
       </x:c>
       <x:c r="E252" s="4" t="n">
-        <x:v>15</x:v>
+        <x:v>180</x:v>
       </x:c>
     </x:row>
     <x:row r="253">
@@ -5518,7 +5518,7 @@
         <x:v>28143</x:v>
       </x:c>
       <x:c r="E253" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>600</x:v>
       </x:c>
     </x:row>
     <x:row r="254">
@@ -5535,7 +5535,7 @@
         <x:v>28144</x:v>
       </x:c>
       <x:c r="E254" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>1200</x:v>
       </x:c>
     </x:row>
     <x:row r="255">
@@ -5552,7 +5552,7 @@
         <x:v>28145</x:v>
       </x:c>
       <x:c r="E255" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>2700</x:v>
       </x:c>
     </x:row>
     <x:row r="256">
@@ -5569,7 +5569,7 @@
         <x:v>28146</x:v>
       </x:c>
       <x:c r="E256" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>3600</x:v>
       </x:c>
     </x:row>
     <x:row r="257">
@@ -5586,7 +5586,7 @@
         <x:v>28147</x:v>
       </x:c>
       <x:c r="E257" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>7200</x:v>
       </x:c>
     </x:row>
     <x:row r="258">
@@ -5603,7 +5603,7 @@
         <x:v>28148</x:v>
       </x:c>
       <x:c r="E258" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>14400</x:v>
       </x:c>
     </x:row>
     <x:row r="259">
@@ -5620,7 +5620,7 @@
         <x:v>28149</x:v>
       </x:c>
       <x:c r="E259" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>28800</x:v>
       </x:c>
     </x:row>
     <x:row r="260">
@@ -5637,7 +5637,7 @@
         <x:v>28150</x:v>
       </x:c>
       <x:c r="E260" s="4" t="n">
-        <x:v>20</x:v>
+        <x:v>43200</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>